<commit_message>
save/load map figure as mat is working
</commit_message>
<xml_diff>
--- a/Docs/MapLab3D_doc.xlsx
+++ b/Docs/MapLab3D_doc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Projekte\MapLab3D\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71CA4D0A-04B5-458C-8951-F95FCD8D942E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B9687E1-2A67-486D-A37D-47989B608198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25740" yWindow="0" windowWidth="25950" windowHeight="20865" tabRatio="836" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27825" yWindow="7605" windowWidth="24075" windowHeight="11295" tabRatio="836" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GV" sheetId="8" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="1296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1968" uniqueCount="1298">
   <si>
     <t>osm</t>
   </si>
@@ -3986,6 +3986,14 @@
   </si>
   <si>
     <t>Axis children is a map object or source plot (true/false). Only needed for saving and loading of the project.</t>
+  </si>
+  <si>
+    <t>GV.openfigureformat</t>
+  </si>
+  <si>
+    <t>Figure format
+old: 'fig' (large figures could no longer be loaded after being saved several times, cause unknown)
+new: 'mat' (starting with version 1.2)</t>
   </si>
 </sst>
 </file>
@@ -10518,7 +10526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:D139"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.85546875" customWidth="1"/>
@@ -11700,203 +11708,203 @@
         <v>1279</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A114" s="23" t="s">
-        <v>383</v>
-      </c>
-      <c r="C114" s="1"/>
+    <row r="113" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B113" t="s">
+        <v>319</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>1297</v>
+      </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C115" s="1"/>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="C116" s="1"/>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" s="23" t="s">
         <v>1027</v>
       </c>
-      <c r="C116" s="1"/>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>562</v>
-      </c>
-      <c r="C117" t="s">
-        <v>564</v>
-      </c>
+      <c r="C117" s="1"/>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C118" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>181</v>
+        <v>563</v>
       </c>
       <c r="C119" t="s">
-        <v>178</v>
+        <v>565</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>1028</v>
+        <v>181</v>
       </c>
       <c r="C120" t="s">
-        <v>1029</v>
+        <v>178</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>1169</v>
+        <v>1028</v>
       </c>
       <c r="C121" t="s">
-        <v>1170</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="C122" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>180</v>
+        <v>1171</v>
       </c>
       <c r="C123" t="s">
-        <v>179</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>180</v>
+      </c>
+      <c r="C124" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
         <v>287</v>
       </c>
-      <c r="C124" t="s">
+      <c r="C125" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A126" s="23" t="s">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" s="23" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>483</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B128" t="s">
         <v>733</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A128" s="36" t="s">
-        <v>450</v>
-      </c>
-      <c r="B128" t="s">
-        <v>81</v>
-      </c>
-      <c r="C128" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="36" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="B129" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C129" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="36" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B130" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C130" t="s">
-        <v>442</v>
+        <v>456</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="36" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B131" t="s">
-        <v>440</v>
+        <v>86</v>
       </c>
       <c r="C131" t="s">
-        <v>378</v>
+        <v>442</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="36" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B132" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="C132" t="s">
-        <v>443</v>
+        <v>378</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="36" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="B133" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C133" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="36" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B134" t="s">
-        <v>163</v>
+        <v>447</v>
       </c>
       <c r="C134" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="36" t="s">
-        <v>511</v>
+        <v>454</v>
       </c>
       <c r="B135" t="s">
-        <v>512</v>
+        <v>163</v>
       </c>
       <c r="C135" t="s">
-        <v>513</v>
+        <v>445</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="36" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="B136" t="s">
-        <v>319</v>
+        <v>512</v>
       </c>
       <c r="C136" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="36" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B137" t="s">
         <v>319</v>
@@ -11907,7 +11915,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="36" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B138" t="s">
         <v>319</v>
@@ -11918,12 +11926,23 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" s="36" t="s">
-        <v>1211</v>
+        <v>516</v>
       </c>
       <c r="B139" t="s">
         <v>319</v>
       </c>
       <c r="C139" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" s="36" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B140" t="s">
+        <v>319</v>
+      </c>
+      <c r="C140" t="s">
         <v>1212</v>
       </c>
     </row>

</xml_diff>